<commit_message>
Refactor bulk_mailer.py to strictly match the 2.3 Python Bulk Mailer Skeleton
</commit_message>
<xml_diff>
--- a/ceo_data.xlsx
+++ b/ceo_data.xlsx
@@ -437,11 +437,11 @@
   <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
@@ -1076,7 +1076,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1094,9 +1094,9 @@
           <t>1,560</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1180,7 +1180,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1198,9 +1198,9 @@
           <t>382,894</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1232,7 +1232,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Koji Sato</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1250,9 +1250,9 @@
           <t>380,793</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>koji.sato@corporate.com</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1302,9 +1302,9 @@
           <t>48,000</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1388,7 +1388,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1406,9 +1406,9 @@
           <t>44,000</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1458,9 +1458,9 @@
           <t>12,479</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1492,7 +1492,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Ron Vachris</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1510,9 +1510,9 @@
           <t>316,000</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>ron.vachris@corporate.com</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1544,7 +1544,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Jamie Dimon</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1562,9 +1562,9 @@
           <t>309,926</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>jamie.dimon@corporate.com</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1700,7 +1700,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1718,9 +1718,9 @@
           <t>36,000</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1804,7 +1804,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1822,9 +1822,9 @@
           <t>47,520</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Carlos Tavares</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1874,9 +1874,9 @@
           <t>258,275</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>carlos.tavares@corporate.com</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1908,7 +1908,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Michael Wirth</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1926,9 +1926,9 @@
           <t>45,600</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>michael.wirth@corporate.com</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1960,7 +1960,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1978,9 +1978,9 @@
           <t>376,871</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2012,7 +2012,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Han Jong-hee</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2030,9 +2030,9 @@
           <t>267,860</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>han.jong-hee@corporate.com</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2064,7 +2064,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>David Cordani</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2082,9 +2082,9 @@
           <t>71,413</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>david.cordani@corporate.com</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2134,9 +2134,9 @@
           <t>451,003</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2168,7 +2168,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2186,9 +2186,9 @@
           <t>595,000</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2220,7 +2220,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2238,9 +2238,9 @@
           <t>314,149</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2272,7 +2272,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2290,9 +2290,9 @@
           <t>160,000</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2324,7 +2324,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Jim Farley</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2342,9 +2342,9 @@
           <t>177,000</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>jim.farley@corporate.com</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2376,7 +2376,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2394,9 +2394,9 @@
           <t>306,931</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Mary Barra</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2446,9 +2446,9 @@
           <t>163,000</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>mary.barra@corporate.com</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2498,9 +2498,9 @@
           <t>104,900</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2532,7 +2532,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2550,9 +2550,9 @@
           <t>154,950</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2584,7 +2584,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2602,9 +2602,9 @@
           <t>166,056</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2688,7 +2688,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2706,9 +2706,9 @@
           <t>336,433</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2740,7 +2740,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2758,9 +2758,9 @@
           <t>258,697</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2792,7 +2792,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2810,9 +2810,9 @@
           <t>237,925</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2844,7 +2844,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2862,9 +2862,9 @@
           <t>China</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2896,7 +2896,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2914,9 +2914,9 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3000,7 +3000,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3014,9 +3014,9 @@
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -3048,7 +3048,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Unknown CEO</t>
+          <t>Search Result (Demo)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3066,9 +3066,9 @@
           <t>Taiwan</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Contact Pending</t>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>search.result.(demo)@corporate.com</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -3108,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3698,27 +3698,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Satya Nadella</t>
+          <t>Koji Sato</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Information technology</t>
+          <t>Automotive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>228,000</t>
+          <t>380,793</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>satya.nadella@corporate.com</t>
+          <t>koji.sato@corporate.com</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=Microsoft%20CEO</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Toyota%20CEO</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>312</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -3750,27 +3750,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Patrick Pouyanné</t>
+          <t>Satya Nadella</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TotalEnergies</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Oil and gas</t>
+          <t>Information technology</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>102,579</t>
+          <t>228,000</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>patrick.pouyanné@corporate.com</t>
+          <t>satya.nadella@corporate.com</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=TotalEnergies%20CEO</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Microsoft%20CEO</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>218</t>
+          <t>281</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -3802,27 +3802,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gary Nagle</t>
+          <t>Ron Vachris</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Glencore</t>
+          <t>Costco</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>83,426</t>
+          <t>316,000</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>gary.nagle@corporate.com</t>
+          <t>ron.vachris@corporate.com</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=Glencore%20CEO</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Costco%20CEO</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>242</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -3854,27 +3854,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Murray Auchincloss</t>
+          <t>Jamie Dimon</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BP</t>
+          <t>JPMorgan Chase</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Oil and gas</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79,400</t>
+          <t>309,926</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>murray.auchincloss@corporate.com</t>
+          <t>jamie.dimon@corporate.com</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=BP%20CEO</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=JPMorgan Chase%20CEO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>239</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -3906,27 +3906,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mark Zuckerberg</t>
+          <t>Patrick Pouyanné</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meta Platforms</t>
+          <t>TotalEnergies</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Social media</t>
+          <t>Oil and gas</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>78,450</t>
+          <t>102,579</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>mark.zuckerberg@corporate.com</t>
+          <t>patrick.pouyanné@corporate.com</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/search/results/all/?keywords=Meta Platforms%20CEO</t>
+          <t>https://www.linkedin.com/search/results/all/?keywords=TotalEnergies%20CEO</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>218</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -3958,50 +3958,518 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Gary Nagle</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Glencore</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Commodities</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>83,426</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>gary.nagle@corporate.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Glencore%20CEO</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Murray Auchincloss</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BP</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Oil and gas</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>79,400</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>murray.auchincloss@corporate.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=BP%20CEO</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Carlos Tavares</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Stellantis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>258,275</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>carlos.tavares@corporate.com</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Stellantis%20CEO</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Michael Wirth</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Oil and gas</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>45,600</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>michael.wirth@corporate.com</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Chevron%20CEO</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Han Jong-hee</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Samsung Electronics</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Electronics</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>267,860</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>han.jong-hee@corporate.com</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Samsung Electronics%20CEO</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>David Cordani</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cigna</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>71,413</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>david.cordani@corporate.com</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Cigna%20CEO</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Jim Farley</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Ford Motor Company</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>177,000</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>jim.farley@corporate.com</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Ford Motor Company%20CEO</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mary Barra</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>General Motors</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>163,000</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>mary.barra@corporate.com</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=General Motors%20CEO</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mark Zuckerberg</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Social media</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>78,450</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>mark.zuckerberg@corporate.com</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/search/results/all/?keywords=Meta Platforms%20CEO</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Hou Qijun</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>China National Petroleum Corporation</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>476</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>hou.qijun@corporate.com</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>+1-XXX-XXX-XXXX (Switchboard)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
         <is>
           <t>https://www.linkedin.com/search/results/all/?keywords=China National Petroleum Corporation%20CEO</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Billionaire Status</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Billionaire Status</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>25.2</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/List_of_largest_companies_by_revenue</t>
         </is>

</xml_diff>